<commit_message>
Incremental deploy (changed files only)
</commit_message>
<xml_diff>
--- a/assets/r02/sheets/空白敵人角色卡.xlsx
+++ b/assets/r02/sheets/空白敵人角色卡.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="敵人角色卡" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCP收容檔案" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,18 +26,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Microsoft JhengHei"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Microsoft JhengHei"/>
       <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
+      <name val="Microsoft JhengHei"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,11 +50,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="008B0000"/>
+        <bgColor rgb="008B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCDCDC"/>
+        <bgColor rgb="00DCDCDC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -58,15 +69,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,161 +455,707 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>敵人角色卡（空白模板）— 參照第4列範例填寫</t>
-        </is>
-      </c>
+          <t>SCP基金會 異常收容檔案</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>基本資料</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>名稱</t>
-        </is>
-      </c>
+          <t>項目編號</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>類型</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Lv</t>
-        </is>
-      </c>
+          <t>項目分級</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>HP(公式)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>ATK</t>
-        </is>
-      </c>
+          <t>收容等級</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>HIT(公式)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>EVA(公式)</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>SPD</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>EXP(公式)</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>特殊/掉落</t>
-        </is>
-      </c>
+          <t>威脅等級(1-5)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>狂暴山豬</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>獸型</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="K4">
-        <f>2*15</f>
-        <v/>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>第1層, 突進</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>別名/暱稱</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>站點位置</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>（角色圖：請貼入或註記圖片路徑）</t>
-        </is>
-      </c>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>戰鬥參數</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HP/耐久</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>迴避(AGI)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>速度(m)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>先攻</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>穿刺DR</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>切割DR</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>鈍擊DR</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>熱力DR</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>化學DR</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>輻射DR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>異常抗性</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>理智光環</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>屬性</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>STR 力量</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>AGI 敏捷</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>END 耐力</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>INT 智力</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>PER 感知</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>WIL 意志</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>__</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>PRE 氣場</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>__</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>特殊能力</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="1" t="n"/>
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="n"/>
+      <c r="H16" s="1" t="n"/>
+      <c r="I16" s="1" t="n"/>
+      <c r="J16" s="1" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>能力名稱</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>觸發條件</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>動作消耗</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>使用頻率</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>範圍</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>效果</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>豁免TN</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>收容協議</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>標準收容措施</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>突破收容緊急協議</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>已知弱點</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>戰術筆記（GM專用）</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>遭遇設計建議</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>建議小隊等級</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>難度預算</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>非戰鬥路徑</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>備註 / 劇情角色</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr"/>
+      <c r="B46" s="3" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr"/>
+      <c r="B47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr"/>
+      <c r="B49" s="3" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A11:J11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>